<commit_message>
Actualizacion diaria del dashboard de inventarios
</commit_message>
<xml_diff>
--- a/bodegas/001.xlsx
+++ b/bodegas/001.xlsx
@@ -431,7 +431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Consolidado (costo desde Existencias Totales) generado el 2026-08-02</t>
+          <t>Consolidado (costo desde Existencias Totales) generado el 2026-07-31</t>
         </is>
       </c>
     </row>
@@ -673,10 +673,10 @@
         <v>587</v>
       </c>
       <c r="N7" t="n">
-        <v>3376.7465268817</v>
+        <v>3376.746528748</v>
       </c>
       <c r="O7" t="n">
-        <v>1982150.211279558</v>
+        <v>1982150.212375076</v>
       </c>
       <c r="P7" t="n">
         <v>4500</v>
@@ -1112,10 +1112,10 @@
         <v>334</v>
       </c>
       <c r="N18" t="n">
-        <v>6272.8539724138</v>
+        <v>6272.8539614856</v>
       </c>
       <c r="O18" t="n">
-        <v>2095133.226786209</v>
+        <v>2095133.22313619</v>
       </c>
       <c r="P18" t="n">
         <v>7900</v>
@@ -1190,10 +1190,10 @@
         <v>450</v>
       </c>
       <c r="N20" t="n">
-        <v>3926.8371355499</v>
+        <v>3926.8371399387</v>
       </c>
       <c r="O20" t="n">
-        <v>1767076.710997455</v>
+        <v>1767076.712972415</v>
       </c>
       <c r="P20" t="n">
         <v>4800</v>
@@ -1388,10 +1388,10 @@
         <v>55</v>
       </c>
       <c r="N25" t="n">
-        <v>12793.680086207</v>
+        <v>12793.680085837</v>
       </c>
       <c r="O25" t="n">
-        <v>703652.404741385</v>
+        <v>703652.404721035</v>
       </c>
       <c r="P25" t="n">
         <v>24000</v>
@@ -1583,10 +1583,10 @@
         <v>62</v>
       </c>
       <c r="N30" t="n">
-        <v>14857.62306383</v>
+        <v>14857.623050847</v>
       </c>
       <c r="O30" t="n">
-        <v>921172.62995746</v>
+        <v>921172.629152514</v>
       </c>
       <c r="P30" t="n">
         <v>34900</v>
@@ -1705,10 +1705,10 @@
         <v>135</v>
       </c>
       <c r="N33" t="n">
-        <v>3910.628317757</v>
+        <v>3910.6283208955</v>
       </c>
       <c r="O33" t="n">
-        <v>527934.822897195</v>
+        <v>527934.8233208925</v>
       </c>
       <c r="P33" t="n">
         <v>9100</v>
@@ -1747,10 +1747,10 @@
         <v>42</v>
       </c>
       <c r="N34" t="n">
-        <v>15711.966441948</v>
+        <v>15711.966494465</v>
       </c>
       <c r="O34" t="n">
-        <v>659902.590561816</v>
+        <v>659902.59276753</v>
       </c>
       <c r="P34" t="n">
         <v>28500</v>
@@ -2500,10 +2500,10 @@
         <v>24</v>
       </c>
       <c r="N52" t="n">
-        <v>4878.2852688172</v>
+        <v>4878.2851851852</v>
       </c>
       <c r="O52" t="n">
-        <v>117078.8464516128</v>
+        <v>117078.8444444448</v>
       </c>
       <c r="P52" t="n">
         <v>13500</v>
@@ -2695,10 +2695,10 @@
         <v>178</v>
       </c>
       <c r="N57" t="n">
-        <v>3340.6800775194</v>
+        <v>3340.6800773694</v>
       </c>
       <c r="O57" t="n">
-        <v>594641.0537984532</v>
+        <v>594641.0537717532</v>
       </c>
       <c r="P57" t="n">
         <v>7100</v>
@@ -2999,10 +2999,10 @@
         <v>228</v>
       </c>
       <c r="N64" t="n">
-        <v>1950.2152617329</v>
+        <v>1950.2152745275</v>
       </c>
       <c r="O64" t="n">
-        <v>444649.0796751012</v>
+        <v>444649.08259227</v>
       </c>
       <c r="P64" t="n">
         <v>2900</v>
@@ -3086,10 +3086,10 @@
         <v>434</v>
       </c>
       <c r="N66" t="n">
-        <v>4937.3101589595</v>
+        <v>4937.3101582734</v>
       </c>
       <c r="O66" t="n">
-        <v>2142792.608988423</v>
+        <v>2142792.608690655</v>
       </c>
       <c r="P66" t="n">
         <v>7500</v>
@@ -3440,10 +3440,10 @@
         <v>120</v>
       </c>
       <c r="N74" t="n">
-        <v>1098.0517240829</v>
+        <v>1098.0510925004</v>
       </c>
       <c r="O74" t="n">
-        <v>131766.206889948</v>
+        <v>131766.131100048</v>
       </c>
       <c r="P74" t="n">
         <v>1500</v>
@@ -4911,10 +4911,10 @@
         <v>577</v>
       </c>
       <c r="N107" t="n">
-        <v>3795.7100070286</v>
+        <v>3795.7100070249</v>
       </c>
       <c r="O107" t="n">
-        <v>2190124.674055502</v>
+        <v>2190124.674053367</v>
       </c>
       <c r="P107" t="n">
         <v>6200</v>
@@ -5843,13 +5843,13 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>198</v>
+        <v>278</v>
       </c>
       <c r="K128" t="n">
         <v>0</v>
       </c>
       <c r="L128" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="M128" t="n">
         <v>198</v>
@@ -6074,10 +6074,10 @@
         <v>535</v>
       </c>
       <c r="N133" t="n">
-        <v>3041.6600119048</v>
+        <v>3041.6600117855</v>
       </c>
       <c r="O133" t="n">
-        <v>1627288.106369068</v>
+        <v>1627288.106305243</v>
       </c>
       <c r="P133" t="n">
         <v>5500</v>
@@ -7659,10 +7659,10 @@
         <v>300</v>
       </c>
       <c r="N168" t="n">
-        <v>1630.9228220183</v>
+        <v>1630.9227791832</v>
       </c>
       <c r="O168" t="n">
-        <v>489276.84660549</v>
+        <v>489276.83375496</v>
       </c>
       <c r="P168" t="n">
         <v>2500</v>
@@ -7705,10 +7705,10 @@
         <v>96</v>
       </c>
       <c r="N169" t="n">
-        <v>1550.1927548066</v>
+        <v>1550.1927149023</v>
       </c>
       <c r="O169" t="n">
-        <v>148818.5044614336</v>
+        <v>148818.5006306208</v>
       </c>
       <c r="P169" t="n">
         <v>2500</v>
@@ -9092,10 +9092,10 @@
         <v>348</v>
       </c>
       <c r="N201" t="n">
-        <v>2029.8734883721</v>
+        <v>2029.8734867503</v>
       </c>
       <c r="O201" t="n">
-        <v>706395.9739534907</v>
+        <v>706395.9733891044</v>
       </c>
       <c r="P201" t="n">
         <v>3600</v>
@@ -9297,10 +9297,10 @@
         <v>170</v>
       </c>
       <c r="N206" t="n">
-        <v>2680.7397012195</v>
+        <v>2680.7397015834</v>
       </c>
       <c r="O206" t="n">
-        <v>455725.749207315</v>
+        <v>455725.749269178</v>
       </c>
       <c r="P206" t="n">
         <v>4900</v>
@@ -9425,10 +9425,10 @@
         <v>237</v>
       </c>
       <c r="N209" t="n">
-        <v>1732.9153957286</v>
+        <v>1732.9154130163</v>
       </c>
       <c r="O209" t="n">
-        <v>410700.9487876782</v>
+        <v>410700.9528848631</v>
       </c>
       <c r="P209" t="n">
         <v>1900</v>
@@ -10806,10 +10806,10 @@
         <v>154</v>
       </c>
       <c r="N241" t="n">
-        <v>548.14729553903</v>
+        <v>548.14741563055</v>
       </c>
       <c r="O241" t="n">
-        <v>84414.68351301062</v>
+        <v>84414.7020071047</v>
       </c>
       <c r="P241" t="n">
         <v>2000</v>
@@ -11939,10 +11939,10 @@
         <v>1215</v>
       </c>
       <c r="N266" t="n">
-        <v>1778.4724932172</v>
+        <v>1778.4724843483</v>
       </c>
       <c r="O266" t="n">
-        <v>2160844.079258898</v>
+        <v>2160844.068483185</v>
       </c>
       <c r="P266" t="n">
         <v>4900</v>
@@ -14253,10 +14253,10 @@
         <v>263</v>
       </c>
       <c r="N316" t="n">
-        <v>2252.2960775371</v>
+        <v>2252.2960568182</v>
       </c>
       <c r="O316" t="n">
-        <v>592353.8683922573</v>
+        <v>592353.8629431867</v>
       </c>
       <c r="P316" t="n">
         <v>3900</v>
@@ -14440,10 +14440,10 @@
         <v>504</v>
       </c>
       <c r="N320" t="n">
-        <v>2328.1187653599</v>
+        <v>2328.1187675234</v>
       </c>
       <c r="O320" t="n">
-        <v>1173371.85774139</v>
+        <v>1173371.858831794</v>
       </c>
       <c r="P320" t="n">
         <v>4500</v>
@@ -14854,10 +14854,10 @@
         <v>184</v>
       </c>
       <c r="N329" t="n">
-        <v>4907.8218731563</v>
+        <v>4907.8218486172</v>
       </c>
       <c r="O329" t="n">
-        <v>903039.2246607592</v>
+        <v>903039.2201455648</v>
       </c>
       <c r="P329" t="n">
         <v>8200</v>
@@ -16321,10 +16321,10 @@
         <v>60</v>
       </c>
       <c r="N361" t="n">
-        <v>4268.7018707483</v>
+        <v>4268.7018305085</v>
       </c>
       <c r="O361" t="n">
-        <v>256122.112244898</v>
+        <v>256122.10983051</v>
       </c>
       <c r="P361" t="n">
         <v>6900</v>
@@ -16827,10 +16827,10 @@
         <v>839</v>
       </c>
       <c r="N372" t="n">
-        <v>1516.0388206553</v>
+        <v>1516.0388215585</v>
       </c>
       <c r="O372" t="n">
-        <v>1271956.570529797</v>
+        <v>1271956.571287582</v>
       </c>
       <c r="P372" t="n">
         <v>2300</v>
@@ -17234,10 +17234,10 @@
         <v>2243</v>
       </c>
       <c r="N381" t="n">
-        <v>692.1519887834301</v>
+        <v>692.15197854077</v>
       </c>
       <c r="O381" t="n">
-        <v>1552496.910841234</v>
+        <v>1552496.887866947</v>
       </c>
       <c r="P381" t="n">
         <v>1200</v>
@@ -18187,10 +18187,10 @@
         <v>238</v>
       </c>
       <c r="N401" t="n">
-        <v>1690.8700087222</v>
+        <v>1690.8700086994</v>
       </c>
       <c r="O401" t="n">
-        <v>402427.0620758836</v>
+        <v>402427.0620704572</v>
       </c>
       <c r="P401" t="n">
         <v>3000</v>
@@ -18471,10 +18471,10 @@
         <v>78</v>
       </c>
       <c r="N407" t="n">
-        <v>3907.5003162055</v>
+        <v>3907.5003137255</v>
       </c>
       <c r="O407" t="n">
-        <v>304785.024664029</v>
+        <v>304785.024470589</v>
       </c>
       <c r="P407" t="n">
         <v>3900</v>
@@ -18564,10 +18564,10 @@
         <v>7734</v>
       </c>
       <c r="N409" t="n">
-        <v>711.33665018328</v>
+        <v>711.33665411716</v>
       </c>
       <c r="O409" t="n">
-        <v>5501477.652517487</v>
+        <v>5501477.682942116</v>
       </c>
       <c r="P409" t="n">
         <v>900</v>
@@ -19216,10 +19216,10 @@
         <v>2</v>
       </c>
       <c r="N423" t="n">
-        <v>3110.8438819661</v>
+        <v>3110.8439531303</v>
       </c>
       <c r="O423" t="n">
-        <v>6221.6877639322</v>
+        <v>6221.6879062606</v>
       </c>
       <c r="P423" t="n">
         <v>4500</v>
@@ -20150,10 +20150,10 @@
         <v>381</v>
       </c>
       <c r="N443" t="n">
-        <v>1595.5196456996</v>
+        <v>1595.5196827833</v>
       </c>
       <c r="O443" t="n">
-        <v>607892.9850115476</v>
+        <v>607892.9991404372</v>
       </c>
       <c r="P443" t="n">
         <v>2500</v>
@@ -22234,10 +22234,10 @@
         <v>152</v>
       </c>
       <c r="N486" t="n">
-        <v>7046.9398310097</v>
+        <v>7046.9398312236</v>
       </c>
       <c r="O486" t="n">
-        <v>1071134.854313474</v>
+        <v>1071134.854345987</v>
       </c>
       <c r="P486" t="n">
         <v>9900</v>
@@ -22332,10 +22332,10 @@
         <v>9</v>
       </c>
       <c r="N488" t="n">
-        <v>15577.048235294</v>
+        <v>15577.047777778</v>
       </c>
       <c r="O488" t="n">
-        <v>140193.434117646</v>
+        <v>140193.430000002</v>
       </c>
       <c r="P488" t="n">
         <v>19900</v>
@@ -22865,10 +22865,10 @@
         <v>70</v>
       </c>
       <c r="N499" t="n">
-        <v>44113.603675676</v>
+        <v>44113.603597884</v>
       </c>
       <c r="O499" t="n">
-        <v>3087952.25729732</v>
+        <v>3087952.25185188</v>
       </c>
       <c r="P499" t="n">
         <v>71900</v>
@@ -23517,10 +23517,10 @@
         <v>216</v>
       </c>
       <c r="N513" t="n">
-        <v>1008.8197488922</v>
+        <v>1008.8200998573</v>
       </c>
       <c r="O513" t="n">
-        <v>217905.0657607152</v>
+        <v>217905.1415691768</v>
       </c>
       <c r="P513" t="n">
         <v>1500</v>
@@ -23820,10 +23820,10 @@
         <v>11</v>
       </c>
       <c r="N520" t="n">
-        <v>22951.705024752</v>
+        <v>22951.705030902</v>
       </c>
       <c r="O520" t="n">
-        <v>252468.755272272</v>
+        <v>252468.755339922</v>
       </c>
       <c r="P520" t="n">
         <v>37900</v>

</xml_diff>